<commit_message>
Version 2.2.2 - Owner reminder and WhatsApp integration
</commit_message>
<xml_diff>
--- a/records/customer_master.xlsx
+++ b/records/customer_master.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ11"/>
+  <dimension ref="A1:AZ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14.453125" bestFit="1" customWidth="1" min="16" max="16"/>
@@ -2574,10 +2574,6 @@
           <t>मुलगा</t>
         </is>
       </c>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
-      <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="inlineStr">
         <is>
           <t>रूम नं: ३०१, नवनाथ सदन, कोपरीगाव 
@@ -2645,7 +2641,871 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="AZ11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>c7f15494</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>वित्तेश मोरे</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>रूम नं: ३०१, नवनाथ सदन, कोपरीगाव
+वाशी सेक्टर २६A, नवी मुंबई</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>९१३७३८३५३५</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2ac49edd</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>वित्तेश मोरे</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>रूम नं: ३०१, नवनाथ सदन, कोपरीगाव
+वाशी सेक्टर २६A, नवी मुंबई</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>९१३७३८३५३५</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2e359608</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2bd6ecd2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>संदीप मोहन पवार</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>3f7dbfee</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R16" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0eeffa0e</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>03c1746c</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>संदीप मोहन पवार</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>d13c7d13</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>संदीप मोहन पवार</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>RSTUV7890P</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R19" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>f85defd5</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>संदीप मोहन पवार</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R20" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>संदीप_मोहन_पवार_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>22ca0fc7</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>मिलिंद अनिल शिंदे</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>7715894705</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>नवनाथ सदन</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>९९८८७७६६५५</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>घर</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>राहण्यासाठी</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>46219</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>नवनाथ_सदन_Rent_Agreement.pdf</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>नवनाथ_सदन_Police_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>